<commit_message>
Estadisticos Primer Parcial 20231 SD
</commit_message>
<xml_diff>
--- a/Totales Generales20231.xlsx
+++ b/Totales Generales20231.xlsx
@@ -602,7 +602,7 @@
         <v>14</v>
       </c>
       <c r="C2">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D2">
         <v>6</v>
@@ -617,10 +617,10 @@
         <v>14</v>
       </c>
       <c r="H2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J2">
         <v>47</v>
@@ -629,10 +629,10 @@
         <v>60</v>
       </c>
       <c r="L2">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="M2" s="1">
-        <v>68.90000000000001</v>
+        <v>69.2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -684,13 +684,13 @@
         <v>14</v>
       </c>
       <c r="C4">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -711,10 +711,10 @@
         <v>21</v>
       </c>
       <c r="L4">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="M4" s="1">
-        <v>88.90000000000001</v>
+        <v>88.8</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -731,7 +731,7 @@
         <v>6</v>
       </c>
       <c r="E5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F5">
         <v>15</v>
@@ -740,10 +740,10 @@
         <v>28</v>
       </c>
       <c r="H5">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I5">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J5">
         <v>236</v>
@@ -766,10 +766,10 @@
         <v>15</v>
       </c>
       <c r="C6">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E6">
         <v>15</v>
@@ -781,10 +781,10 @@
         <v>23</v>
       </c>
       <c r="H6">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I6">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J6">
         <v>24</v>
@@ -793,7 +793,7 @@
         <v>8</v>
       </c>
       <c r="L6">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M6" s="1">
         <v>95.3</v>
@@ -848,13 +848,13 @@
         <v>15</v>
       </c>
       <c r="C8">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F8">
         <v>2</v>
@@ -875,10 +875,10 @@
         <v>35</v>
       </c>
       <c r="L8">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="M8" s="1">
-        <v>70.3</v>
+        <v>69.8</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -889,13 +889,13 @@
         <v>15</v>
       </c>
       <c r="C9">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="D9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E9">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F9">
         <v>32</v>
@@ -904,10 +904,10 @@
         <v>35</v>
       </c>
       <c r="H9">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I9">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J9">
         <v>115</v>
@@ -916,10 +916,10 @@
         <v>89</v>
       </c>
       <c r="L9">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="M9" s="1">
-        <v>79.59999999999999</v>
+        <v>79.5</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -927,13 +927,13 @@
         <v>13</v>
       </c>
       <c r="C10">
-        <v>1040</v>
+        <v>1037</v>
       </c>
       <c r="D10">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E10">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F10">
         <v>47</v>
@@ -954,10 +954,10 @@
         <v>291</v>
       </c>
       <c r="L10">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="M10" s="1">
-        <v>72</v>
+        <v>71.90000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1022,10 +1022,10 @@
         <v>14</v>
       </c>
       <c r="C2">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D2">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -1049,7 +1049,7 @@
         <v>0</v>
       </c>
       <c r="L2">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="M2" s="1">
         <v>100</v>
@@ -1104,13 +1104,13 @@
         <v>14</v>
       </c>
       <c r="C4">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D4">
         <v>56</v>
       </c>
       <c r="E4">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -1131,7 +1131,7 @@
         <v>0</v>
       </c>
       <c r="L4">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="M4" s="1">
         <v>100</v>
@@ -1148,10 +1148,10 @@
         <v>603</v>
       </c>
       <c r="D5">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E5">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -1186,10 +1186,10 @@
         <v>15</v>
       </c>
       <c r="C6">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D6">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1213,7 +1213,7 @@
         <v>0</v>
       </c>
       <c r="L6">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="M6" s="1">
         <v>100</v>
@@ -1268,13 +1268,13 @@
         <v>15</v>
       </c>
       <c r="C8">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D8">
         <v>28</v>
       </c>
       <c r="E8">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -1295,7 +1295,7 @@
         <v>0</v>
       </c>
       <c r="L8">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="M8" s="1">
         <v>100</v>
@@ -1309,13 +1309,13 @@
         <v>15</v>
       </c>
       <c r="C9">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="D9">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E9">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="F9">
         <v>1</v>
@@ -1336,7 +1336,7 @@
         <v>0</v>
       </c>
       <c r="L9">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="M9" s="1">
         <v>100</v>
@@ -1347,13 +1347,13 @@
         <v>13</v>
       </c>
       <c r="C10">
-        <v>1040</v>
+        <v>1037</v>
       </c>
       <c r="D10">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E10">
-        <v>578</v>
+        <v>574</v>
       </c>
       <c r="F10">
         <v>2</v>
@@ -1374,7 +1374,7 @@
         <v>0</v>
       </c>
       <c r="L10">
-        <v>1040</v>
+        <v>1037</v>
       </c>
       <c r="M10" s="1">
         <v>100</v>
@@ -1442,7 +1442,7 @@
         <v>14</v>
       </c>
       <c r="C2">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D2">
         <v>6</v>
@@ -1457,10 +1457,10 @@
         <v>14</v>
       </c>
       <c r="H2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J2">
         <v>47</v>
@@ -1469,10 +1469,10 @@
         <v>60</v>
       </c>
       <c r="L2">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="M2" s="1">
-        <v>68.90000000000001</v>
+        <v>69.2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1524,13 +1524,13 @@
         <v>14</v>
       </c>
       <c r="C4">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -1551,10 +1551,10 @@
         <v>21</v>
       </c>
       <c r="L4">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="M4" s="1">
-        <v>88.90000000000001</v>
+        <v>88.8</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1571,7 +1571,7 @@
         <v>6</v>
       </c>
       <c r="E5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F5">
         <v>15</v>
@@ -1580,10 +1580,10 @@
         <v>28</v>
       </c>
       <c r="H5">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I5">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J5">
         <v>236</v>
@@ -1606,10 +1606,10 @@
         <v>15</v>
       </c>
       <c r="C6">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E6">
         <v>15</v>
@@ -1621,10 +1621,10 @@
         <v>23</v>
       </c>
       <c r="H6">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I6">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J6">
         <v>24</v>
@@ -1633,7 +1633,7 @@
         <v>8</v>
       </c>
       <c r="L6">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M6" s="1">
         <v>95.3</v>
@@ -1688,13 +1688,13 @@
         <v>15</v>
       </c>
       <c r="C8">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F8">
         <v>2</v>
@@ -1715,10 +1715,10 @@
         <v>35</v>
       </c>
       <c r="L8">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="M8" s="1">
-        <v>70.3</v>
+        <v>69.8</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1729,13 +1729,13 @@
         <v>15</v>
       </c>
       <c r="C9">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="D9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E9">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F9">
         <v>32</v>
@@ -1744,10 +1744,10 @@
         <v>35</v>
       </c>
       <c r="H9">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I9">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J9">
         <v>115</v>
@@ -1756,10 +1756,10 @@
         <v>89</v>
       </c>
       <c r="L9">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="M9" s="1">
-        <v>79.59999999999999</v>
+        <v>79.5</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1767,13 +1767,13 @@
         <v>13</v>
       </c>
       <c r="C10">
-        <v>1040</v>
+        <v>1037</v>
       </c>
       <c r="D10">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E10">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F10">
         <v>47</v>
@@ -1794,10 +1794,10 @@
         <v>291</v>
       </c>
       <c r="L10">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="M10" s="1">
-        <v>72</v>
+        <v>71.90000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1932,7 +1932,7 @@
         <v>19</v>
       </c>
       <c r="B4">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -1950,7 +1950,7 @@
         <v>5</v>
       </c>
       <c r="H4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I4">
         <v>8</v>
@@ -1959,10 +1959,10 @@
         <v>14</v>
       </c>
       <c r="K4">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L4" s="1">
-        <v>58.8</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -1970,7 +1970,7 @@
         <v>20</v>
       </c>
       <c r="B5">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -1985,7 +1985,7 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5">
         <v>6</v>
@@ -1997,10 +1997,10 @@
         <v>17</v>
       </c>
       <c r="K5">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="L5" s="1">
-        <v>56.4</v>
+        <v>57.5</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -2426,13 +2426,13 @@
         <v>32</v>
       </c>
       <c r="B17">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C17">
         <v>0</v>
       </c>
       <c r="D17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -2453,7 +2453,7 @@
         <v>0</v>
       </c>
       <c r="K17">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="L17" s="1">
         <v>100</v>
@@ -2578,7 +2578,7 @@
         <v>36</v>
       </c>
       <c r="B21">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -2596,7 +2596,7 @@
         <v>4</v>
       </c>
       <c r="H21">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I21">
         <v>7</v>
@@ -2605,7 +2605,7 @@
         <v>0</v>
       </c>
       <c r="K21">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L21" s="1">
         <v>100</v>
@@ -2616,7 +2616,7 @@
         <v>37</v>
       </c>
       <c r="B22">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C22">
         <v>2</v>
@@ -2631,7 +2631,7 @@
         <v>6</v>
       </c>
       <c r="G22">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H22">
         <v>8</v>
@@ -2643,7 +2643,7 @@
         <v>0</v>
       </c>
       <c r="K22">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L22" s="1">
         <v>100</v>
@@ -2692,10 +2692,10 @@
         <v>39</v>
       </c>
       <c r="B24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -2719,7 +2719,7 @@
         <v>0</v>
       </c>
       <c r="K24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L24" s="1">
         <v>100</v>
@@ -3072,13 +3072,13 @@
         <v>49</v>
       </c>
       <c r="B34">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C34">
         <v>0</v>
       </c>
       <c r="D34">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E34">
         <v>0</v>
@@ -3099,10 +3099,10 @@
         <v>2</v>
       </c>
       <c r="K34">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L34" s="1">
-        <v>85.7</v>
+        <v>83.3</v>
       </c>
     </row>
   </sheetData>
@@ -3201,7 +3201,7 @@
         <v>19</v>
       </c>
       <c r="B4">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C4">
         <v>14</v>
@@ -3213,13 +3213,13 @@
         <v>14</v>
       </c>
       <c r="F4" s="1">
-        <v>41.2</v>
+        <v>40</v>
       </c>
       <c r="G4" s="1">
         <v>0</v>
       </c>
       <c r="H4" s="1">
-        <v>41.2</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -3227,7 +3227,7 @@
         <v>20</v>
       </c>
       <c r="B5">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5">
         <v>17</v>
@@ -3239,13 +3239,13 @@
         <v>17</v>
       </c>
       <c r="F5" s="1">
-        <v>43.6</v>
+        <v>42.5</v>
       </c>
       <c r="G5" s="1">
         <v>0</v>
       </c>
       <c r="H5" s="1">
-        <v>43.6</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -3539,7 +3539,7 @@
         <v>32</v>
       </c>
       <c r="B17">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -3643,7 +3643,7 @@
         <v>36</v>
       </c>
       <c r="B21">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -3669,7 +3669,7 @@
         <v>37</v>
       </c>
       <c r="B22">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -3721,7 +3721,7 @@
         <v>39</v>
       </c>
       <c r="B24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -3981,7 +3981,7 @@
         <v>49</v>
       </c>
       <c r="B34">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C34">
         <v>2</v>
@@ -3993,13 +3993,13 @@
         <v>2</v>
       </c>
       <c r="F34" s="1">
-        <v>14.3</v>
+        <v>16.7</v>
       </c>
       <c r="G34" s="1">
         <v>0</v>
       </c>
       <c r="H34" s="1">
-        <v>14.3</v>
+        <v>16.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Estadisticos Tercer Parcial 7
</commit_message>
<xml_diff>
--- a/Totales Generales20231.xlsx
+++ b/Totales Generales20231.xlsx
@@ -620,10 +620,10 @@
         <v>27</v>
       </c>
       <c r="I2">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K2">
         <v>66</v>
@@ -743,10 +743,10 @@
         <v>43</v>
       </c>
       <c r="I5">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J5">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K5">
         <v>354</v>
@@ -945,10 +945,10 @@
         <v>80</v>
       </c>
       <c r="I10">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J10">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="K10">
         <v>547</v>
@@ -1125,16 +1125,16 @@
         <v>12</v>
       </c>
       <c r="J4">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K4">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="L4">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="M4" s="1">
-        <v>21.3</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1166,16 +1166,16 @@
         <v>42</v>
       </c>
       <c r="J5">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="K5">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="L5">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="M5" s="1">
-        <v>33.9</v>
+        <v>33.6</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1248,16 +1248,16 @@
         <v>11</v>
       </c>
       <c r="J7">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K7">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L7">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="M7" s="1">
-        <v>37.2</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1286,19 +1286,19 @@
         <v>9</v>
       </c>
       <c r="I8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J8">
         <v>29</v>
       </c>
       <c r="K8">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L8">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M8" s="1">
-        <v>48.7</v>
+        <v>47.9</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1327,19 +1327,19 @@
         <v>34</v>
       </c>
       <c r="I9">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J9">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K9">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="L9">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="M9" s="1">
-        <v>57</v>
+        <v>56.6</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1365,19 +1365,19 @@
         <v>68</v>
       </c>
       <c r="I10">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J10">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="K10">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="L10">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="M10" s="1">
-        <v>43.6</v>
+        <v>43.2</v>
       </c>
     </row>
   </sheetData>
@@ -1445,34 +1445,34 @@
         <v>194</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>9</v>
+      </c>
+      <c r="H2">
         <v>6</v>
       </c>
-      <c r="F2">
-        <v>7</v>
-      </c>
-      <c r="G2">
-        <v>12</v>
-      </c>
-      <c r="H2">
-        <v>21</v>
-      </c>
       <c r="I2">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J2">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="K2">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="L2">
-        <v>109</v>
+        <v>76</v>
       </c>
       <c r="M2" s="1">
-        <v>56.2</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1489,31 +1489,31 @@
         <v>0</v>
       </c>
       <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
         <v>2</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
       </c>
       <c r="G3">
         <v>2</v>
       </c>
       <c r="H3">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I3">
+        <v>5</v>
+      </c>
+      <c r="J3">
         <v>15</v>
       </c>
-      <c r="J3">
-        <v>26</v>
-      </c>
       <c r="K3">
-        <v>166</v>
+        <v>190</v>
       </c>
       <c r="L3">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="M3" s="1">
-        <v>25.2</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1527,34 +1527,34 @@
         <v>188</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
         <v>2</v>
       </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>3</v>
-      </c>
-      <c r="I4">
-        <v>12</v>
-      </c>
       <c r="J4">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="K4">
-        <v>150</v>
+        <v>175</v>
       </c>
       <c r="L4">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="M4" s="1">
-        <v>20.2</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1568,34 +1568,34 @@
         <v>604</v>
       </c>
       <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5">
         <v>6</v>
       </c>
-      <c r="E5">
-        <v>9</v>
-      </c>
       <c r="F5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G5">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H5">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="I5">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="J5">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="K5">
-        <v>401</v>
+        <v>483</v>
       </c>
       <c r="L5">
-        <v>203</v>
+        <v>121</v>
       </c>
       <c r="M5" s="1">
-        <v>33.6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1609,34 +1609,34 @@
         <v>170</v>
       </c>
       <c r="D6">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E6">
+        <v>13</v>
+      </c>
+      <c r="F6">
         <v>12</v>
       </c>
-      <c r="F6">
-        <v>19</v>
-      </c>
       <c r="G6">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="H6">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I6">
         <v>21</v>
       </c>
       <c r="J6">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="K6">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="L6">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="M6" s="1">
-        <v>80</v>
+        <v>74.7</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1656,28 +1656,28 @@
         <v>4</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>4</v>
+      </c>
+      <c r="I7">
         <v>3</v>
       </c>
-      <c r="H7">
-        <v>8</v>
-      </c>
-      <c r="I7">
-        <v>11</v>
-      </c>
       <c r="J7">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="K7">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="L7">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="M7" s="1">
-        <v>37.2</v>
+        <v>20.3</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1697,28 +1697,28 @@
         <v>2</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H8">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I8">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="J8">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="K8">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="L8">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="M8" s="1">
-        <v>48.7</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1732,34 +1732,34 @@
         <v>435</v>
       </c>
       <c r="D9">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E9">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F9">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="G9">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="H9">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="I9">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="J9">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="K9">
-        <v>187</v>
+        <v>240</v>
       </c>
       <c r="L9">
-        <v>248</v>
+        <v>195</v>
       </c>
       <c r="M9" s="1">
-        <v>57</v>
+        <v>44.8</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1770,34 +1770,34 @@
         <v>1039</v>
       </c>
       <c r="D10">
+        <v>24</v>
+      </c>
+      <c r="E10">
+        <v>25</v>
+      </c>
+      <c r="F10">
+        <v>21</v>
+      </c>
+      <c r="G10">
         <v>23</v>
       </c>
-      <c r="E10">
-        <v>27</v>
-      </c>
-      <c r="F10">
-        <v>32</v>
-      </c>
-      <c r="G10">
-        <v>46</v>
-      </c>
       <c r="H10">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="I10">
-        <v>88</v>
+        <v>49</v>
       </c>
       <c r="J10">
-        <v>167</v>
+        <v>132</v>
       </c>
       <c r="K10">
-        <v>588</v>
+        <v>723</v>
       </c>
       <c r="L10">
-        <v>451</v>
+        <v>316</v>
       </c>
       <c r="M10" s="1">
-        <v>43.4</v>
+        <v>30.4</v>
       </c>
     </row>
   </sheetData>
@@ -1859,34 +1859,34 @@
         <v>27</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
         <v>2</v>
       </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>4</v>
-      </c>
       <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
         <v>3</v>
       </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
       <c r="I2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="K2">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="L2" s="1">
-        <v>70.40000000000001</v>
+        <v>59.3</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -1900,31 +1900,31 @@
         <v>1</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
         <v>6</v>
       </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>3</v>
-      </c>
       <c r="J3">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K3">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="L3" s="1">
-        <v>66.7</v>
+        <v>58.3</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -1938,31 +1938,31 @@
         <v>2</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G4">
         <v>2</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J4">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L4" s="1">
-        <v>38.2</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -1973,34 +1973,34 @@
         <v>40</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I5">
+        <v>6</v>
+      </c>
+      <c r="J5">
+        <v>30</v>
+      </c>
+      <c r="K5">
         <v>10</v>
       </c>
-      <c r="J5">
-        <v>22</v>
-      </c>
-      <c r="K5">
-        <v>18</v>
-      </c>
       <c r="L5" s="1">
-        <v>45</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -2014,31 +2014,31 @@
         <v>1</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
         <v>3</v>
       </c>
-      <c r="H6">
-        <v>3</v>
-      </c>
-      <c r="I6">
-        <v>12</v>
-      </c>
       <c r="J6">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="K6">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="L6" s="1">
-        <v>53.8</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -2052,31 +2052,31 @@
         <v>0</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J7">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="K7">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="L7" s="1">
-        <v>73.3</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2099,22 +2099,22 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J8">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="K8">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L8" s="1">
-        <v>23.3</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -2128,7 +2128,7 @@
         <v>0</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -2137,22 +2137,22 @@
         <v>0</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H9">
         <v>2</v>
       </c>
       <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>39</v>
+      </c>
+      <c r="K9">
         <v>3</v>
       </c>
-      <c r="J9">
-        <v>34</v>
-      </c>
-      <c r="K9">
-        <v>8</v>
-      </c>
       <c r="L9" s="1">
-        <v>19</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -2175,22 +2175,22 @@
         <v>1</v>
       </c>
       <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
         <v>2</v>
       </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
-      <c r="I10">
+      <c r="J10">
+        <v>31</v>
+      </c>
+      <c r="K10">
         <v>5</v>
       </c>
-      <c r="J10">
-        <v>27</v>
-      </c>
-      <c r="K10">
-        <v>9</v>
-      </c>
       <c r="L10" s="1">
-        <v>25</v>
+        <v>13.9</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -2207,28 +2207,28 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11">
         <v>0</v>
       </c>
       <c r="G11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H11">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I11">
         <v>5</v>
       </c>
       <c r="J11">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="K11">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="L11" s="1">
-        <v>36.4</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -2248,25 +2248,25 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I12">
         <v>3</v>
       </c>
       <c r="J12">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K12">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L12" s="1">
-        <v>21.9</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -2286,25 +2286,25 @@
         <v>1</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
         <v>3</v>
       </c>
-      <c r="I13">
-        <v>4</v>
-      </c>
       <c r="J13">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="K13">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="L13" s="1">
-        <v>23.7</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -2327,22 +2327,22 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J14">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="K14">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L14" s="1">
-        <v>26.7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -2371,16 +2371,16 @@
         <v>0</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J15">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="K15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L15" s="1">
-        <v>5.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -2397,7 +2397,7 @@
         <v>1</v>
       </c>
       <c r="E16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -2409,16 +2409,16 @@
         <v>1</v>
       </c>
       <c r="I16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J16">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="K16">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L16" s="1">
-        <v>24</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -2447,16 +2447,16 @@
         <v>0</v>
       </c>
       <c r="I17">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J17">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="K17">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L17" s="1">
-        <v>16.1</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -2467,34 +2467,34 @@
         <v>28</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18">
         <v>0</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18">
         <v>0</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J18">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="K18">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L18" s="1">
-        <v>28.6</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -2520,19 +2520,19 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I19">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J19">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="K19">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L19" s="1">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -2543,34 +2543,34 @@
         <v>36</v>
       </c>
       <c r="C20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E20">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G20">
         <v>4</v>
       </c>
       <c r="H20">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J20">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K20">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="L20" s="1">
-        <v>80.59999999999999</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -2581,34 +2581,34 @@
         <v>39</v>
       </c>
       <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>4</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
         <v>2</v>
       </c>
-      <c r="D21">
-        <v>1</v>
-      </c>
-      <c r="E21">
+      <c r="G21">
+        <v>6</v>
+      </c>
+      <c r="H21">
         <v>4</v>
       </c>
-      <c r="F21">
-        <v>6</v>
-      </c>
-      <c r="G21">
-        <v>5</v>
-      </c>
-      <c r="H21">
-        <v>5</v>
-      </c>
       <c r="I21">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J21">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="K21">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="L21" s="1">
-        <v>79.5</v>
+        <v>61.5</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -2619,34 +2619,34 @@
         <v>39</v>
       </c>
       <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22">
+        <v>3</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
+        <v>3</v>
+      </c>
+      <c r="G22">
+        <v>4</v>
+      </c>
+      <c r="H22">
+        <v>8</v>
+      </c>
+      <c r="I22">
+        <v>12</v>
+      </c>
+      <c r="J22">
         <v>5</v>
       </c>
-      <c r="D22">
-        <v>2</v>
-      </c>
-      <c r="E22">
-        <v>4</v>
-      </c>
-      <c r="F22">
-        <v>6</v>
-      </c>
-      <c r="G22">
-        <v>3</v>
-      </c>
-      <c r="H22">
-        <v>4</v>
-      </c>
-      <c r="I22">
-        <v>8</v>
-      </c>
-      <c r="J22">
-        <v>7</v>
-      </c>
       <c r="K22">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L22" s="1">
-        <v>82.09999999999999</v>
+        <v>87.2</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -2657,25 +2657,25 @@
         <v>37</v>
       </c>
       <c r="C23">
+        <v>4</v>
+      </c>
+      <c r="D23">
+        <v>4</v>
+      </c>
+      <c r="E23">
         <v>5</v>
       </c>
-      <c r="D23">
+      <c r="F23">
         <v>3</v>
       </c>
-      <c r="E23">
-        <v>4</v>
-      </c>
-      <c r="F23">
-        <v>9</v>
-      </c>
       <c r="G23">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I23">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J23">
         <v>6</v>
@@ -2695,34 +2695,34 @@
         <v>19</v>
       </c>
       <c r="C24">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D24">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E24">
         <v>1</v>
       </c>
       <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
         <v>2</v>
       </c>
-      <c r="G24">
-        <v>3</v>
-      </c>
       <c r="H24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I24">
         <v>2</v>
       </c>
       <c r="J24">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K24">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L24" s="1">
-        <v>68.40000000000001</v>
+        <v>57.9</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -2745,22 +2745,22 @@
         <v>0</v>
       </c>
       <c r="G25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H25">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I25">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="J25">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="K25">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="L25" s="1">
-        <v>64</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -2774,31 +2774,31 @@
         <v>0</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H26">
         <v>2</v>
       </c>
       <c r="I26">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J26">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="K26">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="L26" s="1">
-        <v>43.9</v>
+        <v>22</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -2815,19 +2815,19 @@
         <v>0</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27">
         <v>2</v>
       </c>
-      <c r="G27">
-        <v>1</v>
-      </c>
       <c r="H27">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I27">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J27">
         <v>16</v>
@@ -2850,7 +2850,7 @@
         <v>0</v>
       </c>
       <c r="D28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -2862,19 +2862,19 @@
         <v>1</v>
       </c>
       <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
         <v>3</v>
       </c>
-      <c r="I28">
-        <v>2</v>
-      </c>
       <c r="J28">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="K28">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L28" s="1">
-        <v>29.6</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -2897,22 +2897,22 @@
         <v>0</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29">
         <v>0</v>
       </c>
       <c r="I29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J29">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="K29">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L29" s="1">
-        <v>13.3</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -2938,19 +2938,19 @@
         <v>1</v>
       </c>
       <c r="H30">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J30">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K30">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L30" s="1">
-        <v>39.3</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -2970,25 +2970,25 @@
         <v>0</v>
       </c>
       <c r="F31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H31">
         <v>3</v>
       </c>
       <c r="I31">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="J31">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="K31">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="L31" s="1">
-        <v>54.5</v>
+        <v>30.3</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -3011,22 +3011,22 @@
         <v>0</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H32">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I32">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J32">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="K32">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L32" s="1">
-        <v>58.8</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -3043,28 +3043,28 @@
         <v>0</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33">
         <v>0</v>
       </c>
       <c r="G33">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H33">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I33">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J33">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="K33">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="L33" s="1">
-        <v>46.2</v>
+        <v>34.6</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -3087,22 +3087,22 @@
         <v>0</v>
       </c>
       <c r="G34">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H34">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I34">
         <v>1</v>
       </c>
       <c r="J34">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K34">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L34" s="1">
-        <v>46.2</v>
+        <v>38.5</v>
       </c>
     </row>
   </sheetData>
@@ -3158,7 +3158,7 @@
         <v>8</v>
       </c>
       <c r="E2">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F2" s="1">
         <v>33.3</v>
@@ -3167,7 +3167,7 @@
         <v>29.6</v>
       </c>
       <c r="H2" s="1">
-        <v>29.6</v>
+        <v>40.7</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -3184,7 +3184,7 @@
         <v>8</v>
       </c>
       <c r="E3">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F3" s="1">
         <v>33.3</v>
@@ -3193,7 +3193,7 @@
         <v>33.3</v>
       </c>
       <c r="H3" s="1">
-        <v>33.3</v>
+        <v>41.7</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -3210,7 +3210,7 @@
         <v>21</v>
       </c>
       <c r="E4">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F4" s="1">
         <v>41.2</v>
@@ -3219,7 +3219,7 @@
         <v>61.8</v>
       </c>
       <c r="H4" s="1">
-        <v>61.8</v>
+        <v>67.59999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -3236,7 +3236,7 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F5" s="1">
         <v>42.5</v>
@@ -3245,7 +3245,7 @@
         <v>55</v>
       </c>
       <c r="H5" s="1">
-        <v>55</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -3262,7 +3262,7 @@
         <v>18</v>
       </c>
       <c r="E6">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F6" s="1">
         <v>30.8</v>
@@ -3271,7 +3271,7 @@
         <v>46.2</v>
       </c>
       <c r="H6" s="1">
-        <v>46.2</v>
+        <v>74.40000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -3288,7 +3288,7 @@
         <v>8</v>
       </c>
       <c r="E7">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F7" s="1">
         <v>20</v>
@@ -3297,7 +3297,7 @@
         <v>26.7</v>
       </c>
       <c r="H7" s="1">
-        <v>26.7</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -3314,7 +3314,7 @@
         <v>23</v>
       </c>
       <c r="E8">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F8" s="1">
         <v>70</v>
@@ -3323,7 +3323,7 @@
         <v>76.7</v>
       </c>
       <c r="H8" s="1">
-        <v>76.7</v>
+        <v>93.3</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -3340,7 +3340,7 @@
         <v>34</v>
       </c>
       <c r="E9">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F9" s="1">
         <v>76.2</v>
@@ -3349,7 +3349,7 @@
         <v>81</v>
       </c>
       <c r="H9" s="1">
-        <v>81</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -3366,7 +3366,7 @@
         <v>27</v>
       </c>
       <c r="E10">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F10" s="1">
         <v>66.7</v>
@@ -3375,7 +3375,7 @@
         <v>75</v>
       </c>
       <c r="H10" s="1">
-        <v>75</v>
+        <v>86.09999999999999</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -3392,7 +3392,7 @@
         <v>28</v>
       </c>
       <c r="E11">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F11" s="1">
         <v>61.4</v>
@@ -3401,7 +3401,7 @@
         <v>63.6</v>
       </c>
       <c r="H11" s="1">
-        <v>63.6</v>
+        <v>70.5</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -3418,7 +3418,7 @@
         <v>25</v>
       </c>
       <c r="E12">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F12" s="1">
         <v>37.5</v>
@@ -3427,7 +3427,7 @@
         <v>78.09999999999999</v>
       </c>
       <c r="H12" s="1">
-        <v>78.09999999999999</v>
+        <v>87.5</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -3444,7 +3444,7 @@
         <v>29</v>
       </c>
       <c r="E13">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F13" s="1">
         <v>73.7</v>
@@ -3453,7 +3453,7 @@
         <v>76.3</v>
       </c>
       <c r="H13" s="1">
-        <v>76.3</v>
+        <v>86.8</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -3467,19 +3467,19 @@
         <v>20</v>
       </c>
       <c r="D14">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E14">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="F14" s="1">
         <v>66.7</v>
       </c>
       <c r="G14" s="1">
-        <v>66.7</v>
+        <v>73.3</v>
       </c>
       <c r="H14" s="1">
-        <v>73.3</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -3496,7 +3496,7 @@
         <v>36</v>
       </c>
       <c r="E15">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F15" s="1">
         <v>94.7</v>
@@ -3505,7 +3505,7 @@
         <v>94.7</v>
       </c>
       <c r="H15" s="1">
-        <v>94.7</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -3522,7 +3522,7 @@
         <v>19</v>
       </c>
       <c r="E16">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F16" s="1">
         <v>80</v>
@@ -3531,7 +3531,7 @@
         <v>76</v>
       </c>
       <c r="H16" s="1">
-        <v>76</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -3548,7 +3548,7 @@
         <v>26</v>
       </c>
       <c r="E17">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F17" s="1">
         <v>74.2</v>
@@ -3557,7 +3557,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="H17" s="1">
-        <v>83.90000000000001</v>
+        <v>96.8</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -3574,7 +3574,7 @@
         <v>20</v>
       </c>
       <c r="E18">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F18" s="1">
         <v>71.40000000000001</v>
@@ -3583,7 +3583,7 @@
         <v>71.40000000000001</v>
       </c>
       <c r="H18" s="1">
-        <v>71.40000000000001</v>
+        <v>78.59999999999999</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -3600,7 +3600,7 @@
         <v>27</v>
       </c>
       <c r="E19">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="F19" s="1">
         <v>69.40000000000001</v>
@@ -3609,7 +3609,7 @@
         <v>75</v>
       </c>
       <c r="H19" s="1">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -3626,7 +3626,7 @@
         <v>7</v>
       </c>
       <c r="E20">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F20" s="1">
         <v>22.2</v>
@@ -3635,7 +3635,7 @@
         <v>19.4</v>
       </c>
       <c r="H20" s="1">
-        <v>19.4</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -3652,7 +3652,7 @@
         <v>8</v>
       </c>
       <c r="E21">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F21" s="1">
         <v>15.4</v>
@@ -3661,7 +3661,7 @@
         <v>20.5</v>
       </c>
       <c r="H21" s="1">
-        <v>20.5</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -3678,7 +3678,7 @@
         <v>7</v>
       </c>
       <c r="E22">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F22" s="1">
         <v>28.2</v>
@@ -3687,7 +3687,7 @@
         <v>17.9</v>
       </c>
       <c r="H22" s="1">
-        <v>17.9</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -3730,7 +3730,7 @@
         <v>6</v>
       </c>
       <c r="E24">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F24" s="1">
         <v>36.8</v>
@@ -3739,7 +3739,7 @@
         <v>31.6</v>
       </c>
       <c r="H24" s="1">
-        <v>31.6</v>
+        <v>42.1</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -3753,19 +3753,19 @@
         <v>12</v>
       </c>
       <c r="D25">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E25">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F25" s="1">
         <v>48</v>
       </c>
       <c r="G25" s="1">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H25" s="1">
-        <v>36</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -3782,7 +3782,7 @@
         <v>23</v>
       </c>
       <c r="E26">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="F26" s="1">
         <v>63.4</v>
@@ -3791,7 +3791,7 @@
         <v>56.1</v>
       </c>
       <c r="H26" s="1">
-        <v>56.1</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -3834,7 +3834,7 @@
         <v>19</v>
       </c>
       <c r="E28">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F28" s="1">
         <v>66.7</v>
@@ -3843,7 +3843,7 @@
         <v>70.40000000000001</v>
       </c>
       <c r="H28" s="1">
-        <v>70.40000000000001</v>
+        <v>81.5</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -3860,7 +3860,7 @@
         <v>26</v>
       </c>
       <c r="E29">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F29" s="1">
         <v>86.7</v>
@@ -3869,7 +3869,7 @@
         <v>86.7</v>
       </c>
       <c r="H29" s="1">
-        <v>86.7</v>
+        <v>93.3</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -3886,7 +3886,7 @@
         <v>17</v>
       </c>
       <c r="E30">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F30" s="1">
         <v>64.3</v>
@@ -3895,7 +3895,7 @@
         <v>60.7</v>
       </c>
       <c r="H30" s="1">
-        <v>60.7</v>
+        <v>64.3</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -3912,7 +3912,7 @@
         <v>15</v>
       </c>
       <c r="E31">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F31" s="1">
         <v>42.4</v>
@@ -3921,7 +3921,7 @@
         <v>45.5</v>
       </c>
       <c r="H31" s="1">
-        <v>45.5</v>
+        <v>69.7</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -3938,7 +3938,7 @@
         <v>7</v>
       </c>
       <c r="E32">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F32" s="1">
         <v>47.1</v>
@@ -3947,7 +3947,7 @@
         <v>41.2</v>
       </c>
       <c r="H32" s="1">
-        <v>41.2</v>
+        <v>76.5</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -3961,19 +3961,19 @@
         <v>19</v>
       </c>
       <c r="D33">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E33">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F33" s="1">
         <v>73.09999999999999</v>
       </c>
       <c r="G33" s="1">
-        <v>53.8</v>
+        <v>57.7</v>
       </c>
       <c r="H33" s="1">
-        <v>53.8</v>
+        <v>65.40000000000001</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -3990,7 +3990,7 @@
         <v>7</v>
       </c>
       <c r="E34">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F34" s="1">
         <v>15.4</v>
@@ -3999,7 +3999,7 @@
         <v>53.8</v>
       </c>
       <c r="H34" s="1">
-        <v>53.8</v>
+        <v>61.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>